<commit_message>
fixed power calculation; changed from relative vbus units to volts; found possible issue in current measuring/voltage pwm generation pins
</commit_message>
<xml_diff>
--- a/Utilities/calcule.xlsx
+++ b/Utilities/calcule.xlsx
@@ -5,16 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marco\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marco\Documents\GitHub\Licenta\Utilities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1529E854-9A9B-46F3-B31A-9E44063C451B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EFF5DAB-E951-4E44-8057-9E9CEEB6F7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F62BF15F-CFC1-4998-96FD-1AE5B823C7CF}"/>
+    <workbookView xWindow="1860" yWindow="1755" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{F62BF15F-CFC1-4998-96FD-1AE5B823C7CF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Saturatie senzor curent" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
   <si>
     <t>rezistenta shunt</t>
   </si>
@@ -54,13 +56,64 @@
     <t>maxim unitati adc</t>
   </si>
   <si>
-    <t>tensiune shunt amplificata</t>
-  </si>
-  <si>
-    <t>tensiune shunt efectiva</t>
-  </si>
-  <si>
-    <t>curent shunt efectiv</t>
+    <t>Valoare osciloscop</t>
+  </si>
+  <si>
+    <t>Valoare ADC</t>
+  </si>
+  <si>
+    <t>Sursa</t>
+  </si>
+  <si>
+    <t>Curent</t>
+  </si>
+  <si>
+    <t>Duty cycle B</t>
+  </si>
+  <si>
+    <t>Duty cycle A</t>
+  </si>
+  <si>
+    <t>Duty cycle C</t>
+  </si>
+  <si>
+    <t>Tensiune</t>
+  </si>
+  <si>
+    <t>24V</t>
+  </si>
+  <si>
+    <t>tensiune șunt amplificata</t>
+  </si>
+  <si>
+    <t>tensiune șunt originală</t>
+  </si>
+  <si>
+    <t>curent șunt</t>
+  </si>
+  <si>
+    <t>Factor amplificare</t>
+  </si>
+  <si>
+    <t>Ia</t>
+  </si>
+  <si>
+    <t>Ib</t>
+  </si>
+  <si>
+    <t>Ic</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>abaterea</t>
   </si>
 </sst>
 </file>
@@ -619,13 +672,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36F02A6E-8B79-423E-820B-C5451F56AE38}">
-  <dimension ref="A2:B9"/>
+  <dimension ref="A2:D9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -633,7 +686,7 @@
         <v>5.0000000000000001E-4</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -641,23 +694,23 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4">
-        <v>610</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5">
-        <v>3.3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -665,31 +718,326 @@
         <v>4095</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="B7">
         <f>B4*B5/B6</f>
-        <v>0.49157509157509155</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.36630036630036628</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B8">
         <f>B7/B3</f>
-        <v>6.1446886446886442E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>4.5787545787545781E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B9">
         <f>B8/B2</f>
-        <v>12.289377289377288</v>
+        <v>9.1575091575091552</v>
+      </c>
+      <c r="C9">
+        <v>2.7359999999999998</v>
+      </c>
+      <c r="D9">
+        <f>C9*B9</f>
+        <v>25.054945054945048</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3190CC9-FDAB-4116-BDE6-C0992EBEA208}">
+  <dimension ref="A2:H15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>4095</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>6.05</v>
+      </c>
+      <c r="C5">
+        <v>5.4</v>
+      </c>
+      <c r="D5">
+        <v>4.38</v>
+      </c>
+      <c r="E5">
+        <v>3.73</v>
+      </c>
+      <c r="F5">
+        <v>3.05</v>
+      </c>
+      <c r="G5">
+        <v>1.95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>360</v>
+      </c>
+      <c r="C6">
+        <v>310</v>
+      </c>
+      <c r="D6">
+        <v>270</v>
+      </c>
+      <c r="E6">
+        <v>225</v>
+      </c>
+      <c r="F6">
+        <v>171</v>
+      </c>
+      <c r="G6">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <f>B3/B4</f>
+        <v>8.0586080586080586E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9">
+        <f>C5/C6</f>
+        <v>1.741935483870968E-2</v>
+      </c>
+      <c r="C9">
+        <f>B5/B6</f>
+        <v>1.6805555555555556E-2</v>
+      </c>
+      <c r="D9">
+        <f t="shared" ref="C9:H9" si="0">D5/D6</f>
+        <v>1.6222222222222221E-2</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>1.6577777777777778E-2</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>1.7836257309941518E-2</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="0"/>
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="H9">
+        <f>AVERAGE(B9:G9)</f>
+        <v>1.6643527950701127E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12">
+        <v>7.6</v>
+      </c>
+      <c r="C12">
+        <f>50+B12</f>
+        <v>57.6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13">
+        <f>B12/2</f>
+        <v>3.8</v>
+      </c>
+      <c r="C13">
+        <f>50-B13</f>
+        <v>46.2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14">
+        <f>B12/2</f>
+        <v>3.8</v>
+      </c>
+      <c r="C14">
+        <f>50-B14</f>
+        <v>46.2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B15">
+        <f>B12+B13</f>
+        <v>11.399999999999999</v>
+      </c>
+      <c r="C15">
+        <v>24</v>
+      </c>
+      <c r="D15">
+        <f>B15*C15/100</f>
+        <v>2.7359999999999998</v>
+      </c>
+      <c r="E15">
+        <v>7.13</v>
+      </c>
+      <c r="F15">
+        <f>E15*D15</f>
+        <v>19.507679999999997</v>
+      </c>
+      <c r="G15">
+        <f>F15*107/100</f>
+        <v>20.873217599999997</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AD61257-B7C9-4F84-AC0E-362CD6DA38E8}">
+  <dimension ref="A2:D14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7">
+        <v>2.8</v>
+      </c>
+      <c r="D7">
+        <v>2.7970000000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8">
+        <v>5.4</v>
+      </c>
+      <c r="D8">
+        <v>5.3819999999999997</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9">
+        <v>2.8</v>
+      </c>
+      <c r="D9">
+        <f>D8/2</f>
+        <v>2.6909999999999998</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10">
+        <f>D8-2*D7</f>
+        <v>-0.21200000000000063</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modified PI values + documentation update
</commit_message>
<xml_diff>
--- a/Utilities/calcule.xlsx
+++ b/Utilities/calcule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marco\Documents\GitHub\Licenta\Utilities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EFF5DAB-E951-4E44-8057-9E9CEEB6F7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB4024CB-9D9F-4D45-BA5F-7CACC16EBEBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="1755" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{F62BF15F-CFC1-4998-96FD-1AE5B823C7CF}"/>
+    <workbookView xWindow="1860" yWindow="1755" windowWidth="18180" windowHeight="11295" activeTab="1" xr2:uid="{F62BF15F-CFC1-4998-96FD-1AE5B823C7CF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
   <si>
     <t>rezistenta shunt</t>
   </si>
@@ -114,6 +114,9 @@
   </si>
   <si>
     <t>abaterea</t>
+  </si>
+  <si>
+    <t>u=ir</t>
   </si>
 </sst>
 </file>
@@ -672,13 +675,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36F02A6E-8B79-423E-820B-C5451F56AE38}">
-  <dimension ref="A2:D9"/>
+  <dimension ref="A2:F11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -686,7 +689,7 @@
         <v>5.0000000000000001E-4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -694,7 +697,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -702,7 +705,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -710,7 +713,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -718,7 +721,7 @@
         <v>4095</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -726,8 +729,11 @@
         <f>B4*B5/B6</f>
         <v>0.36630036630036628</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -736,7 +742,7 @@
         <v>4.5787545787545781E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -750,6 +756,25 @@
       <c r="D9">
         <f>C9*B9</f>
         <v>25.054945054945048</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B10">
+        <f>B9/B4</f>
+        <v>1.8315018315018309E-2</v>
+      </c>
+      <c r="C10">
+        <v>1.6500000000000001E-2</v>
+      </c>
+      <c r="D10">
+        <f>B10-C10</f>
+        <v>1.8150183150183082E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D11">
+        <f>D10/B10</f>
+        <v>9.9099999999999661E-2</v>
       </c>
     </row>
   </sheetData>
@@ -795,22 +820,22 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>6.05</v>
+        <v>1.47</v>
       </c>
       <c r="C5">
+        <v>1.95</v>
+      </c>
+      <c r="D5">
+        <v>3.1</v>
+      </c>
+      <c r="E5">
+        <v>3.71</v>
+      </c>
+      <c r="F5">
+        <v>4.3499999999999996</v>
+      </c>
+      <c r="G5">
         <v>5.4</v>
-      </c>
-      <c r="D5">
-        <v>4.38</v>
-      </c>
-      <c r="E5">
-        <v>3.73</v>
-      </c>
-      <c r="F5">
-        <v>3.05</v>
-      </c>
-      <c r="G5">
-        <v>1.95</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -818,22 +843,22 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>360</v>
+        <v>89</v>
       </c>
       <c r="C6">
-        <v>310</v>
+        <v>130</v>
       </c>
       <c r="D6">
-        <v>270</v>
+        <v>175</v>
       </c>
       <c r="E6">
         <v>225</v>
       </c>
       <c r="F6">
-        <v>171</v>
+        <v>267</v>
       </c>
       <c r="G6">
-        <v>130</v>
+        <v>313</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -858,32 +883,32 @@
         <v>17</v>
       </c>
       <c r="B9">
+        <f>B5/B6</f>
+        <v>1.6516853932584268E-2</v>
+      </c>
+      <c r="C9">
         <f>C5/C6</f>
-        <v>1.741935483870968E-2</v>
-      </c>
-      <c r="C9">
-        <f>B5/B6</f>
-        <v>1.6805555555555556E-2</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="D9">
-        <f t="shared" ref="C9:H9" si="0">D5/D6</f>
-        <v>1.6222222222222221E-2</v>
+        <f>D5/D6</f>
+        <v>1.7714285714285714E-2</v>
       </c>
       <c r="E9">
-        <f t="shared" si="0"/>
-        <v>1.6577777777777778E-2</v>
+        <f>E5/E6</f>
+        <v>1.648888888888889E-2</v>
       </c>
       <c r="F9">
-        <f t="shared" si="0"/>
-        <v>1.7836257309941518E-2</v>
+        <f t="shared" ref="D9:G9" si="0">F5/F6</f>
+        <v>1.6292134831460674E-2</v>
       </c>
       <c r="G9">
         <f t="shared" si="0"/>
-        <v>1.4999999999999999E-2</v>
+        <v>1.7252396166134186E-2</v>
       </c>
       <c r="H9">
         <f>AVERAGE(B9:G9)</f>
-        <v>1.6643527950701127E-2</v>
+        <v>1.6544093255558955E-2</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>